<commit_message>
changed and personalised map pins
</commit_message>
<xml_diff>
--- a/src/data/database_projects.xlsx
+++ b/src/data/database_projects.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Valerie\Documents\uni\Uni Lausanne\SP26\géovisualisation\projet\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76CC40C4-71B8-4DAA-9BF4-FE0F09D8C718}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72EE397B-5BBA-442D-8710-B7CF7D4E49DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="40920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13276" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="projects sportsanddev" sheetId="3" r:id="rId1"/>
@@ -68,21 +68,12 @@
     <t>Asia</t>
   </si>
   <si>
-    <t>Australia</t>
-  </si>
-  <si>
-    <t>Central America</t>
-  </si>
-  <si>
     <t>Europe</t>
   </si>
   <si>
     <t>Latin America and the Caribbean</t>
   </si>
   <si>
-    <t>The Middle East</t>
-  </si>
-  <si>
     <t>North America</t>
   </si>
   <si>
@@ -92,9 +83,6 @@
     <t>Non-profit organization</t>
   </si>
   <si>
-    <t>Sports structure</t>
-  </si>
-  <si>
     <t>Educational structure</t>
   </si>
   <si>
@@ -104,18 +92,12 @@
     <t>country</t>
   </si>
   <si>
-    <t>Refugee context</t>
-  </si>
-  <si>
     <t>Gender equality</t>
   </si>
   <si>
     <t>Youth development</t>
   </si>
   <si>
-    <t>Disability</t>
-  </si>
-  <si>
     <t>Health</t>
   </si>
   <si>
@@ -164,12 +146,6 @@
     <t>People with disabilities</t>
   </si>
   <si>
-    <t>Volunteers</t>
-  </si>
-  <si>
-    <t>Employment</t>
-  </si>
-  <si>
     <t>The football foundation for Africa</t>
   </si>
   <si>
@@ -374,9 +350,6 @@
     <t>Foundation</t>
   </si>
   <si>
-    <t>UN agenca</t>
-  </si>
-  <si>
     <t>Football</t>
   </si>
   <si>
@@ -419,9 +392,6 @@
     <t>Leadership</t>
   </si>
   <si>
-    <t>None</t>
-  </si>
-  <si>
     <t>English</t>
   </si>
   <si>
@@ -474,6 +444,36 @@
   </si>
   <si>
     <t>coaching</t>
+  </si>
+  <si>
+    <t>No prerequisite skills</t>
+  </si>
+  <si>
+    <t>Forced displacement settings</t>
+  </si>
+  <si>
+    <t>Construction work</t>
+  </si>
+  <si>
+    <t>UN agency</t>
+  </si>
+  <si>
+    <t>Sports structure or club</t>
+  </si>
+  <si>
+    <t>1-3 weeks</t>
+  </si>
+  <si>
+    <t>1-3 months</t>
+  </si>
+  <si>
+    <t>4-6 months</t>
+  </si>
+  <si>
+    <t>1 year</t>
+  </si>
+  <si>
+    <t>Flexible</t>
   </si>
 </sst>
 </file>
@@ -538,13 +538,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -834,282 +833,282 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -1137,10 +1136,10 @@
   <sheetData>
     <row r="1" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>6</v>
@@ -1149,43 +1148,43 @@
         <v>7</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>8</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="L1" s="4" t="s">
         <v>4</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="N1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.45">
@@ -1193,7 +1192,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="C2">
         <v>-1.2833300000000001</v>
@@ -1202,43 +1201,43 @@
         <v>36.816670000000002</v>
       </c>
       <c r="E2" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="F2" t="s">
         <v>11</v>
       </c>
       <c r="G2" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="H2" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="I2" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="J2" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="K2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="L2" t="s">
-        <v>104</v>
-      </c>
-      <c r="M2" s="5" t="s">
-        <v>148</v>
+        <v>96</v>
+      </c>
+      <c r="M2" t="s">
+        <v>138</v>
       </c>
       <c r="N2" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="O2" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="Q2" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.45">
@@ -1358,7 +1357,7 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.45">
       <c r="C30" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1371,7 +1370,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B55723D-BFAA-4607-A22F-0BB892FF6917}">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="26.1328125" customWidth="1"/>
@@ -1379,7 +1378,7 @@
     <col min="3" max="3" width="20.73046875" customWidth="1"/>
     <col min="4" max="4" width="15.19921875" customWidth="1"/>
     <col min="5" max="5" width="32.1328125" customWidth="1"/>
-    <col min="6" max="6" width="17.33203125" customWidth="1"/>
+    <col min="6" max="6" width="27.06640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.45">
@@ -1410,207 +1409,205 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>140</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="E2" t="s">
         <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="G2" t="s">
-        <v>131</v>
+        <v>121</v>
+      </c>
+      <c r="H2" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="C3" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="D3" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="E3" t="s">
         <v>11</v>
       </c>
       <c r="F3" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="G3" t="s">
-        <v>132</v>
+        <v>122</v>
+      </c>
+      <c r="H3" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>143</v>
       </c>
       <c r="D4" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="E4" t="s">
         <v>12</v>
       </c>
       <c r="F4" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="G4" t="s">
-        <v>133</v>
+        <v>123</v>
+      </c>
+      <c r="H4" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="E5" t="s">
         <v>13</v>
       </c>
       <c r="F5" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="G5" t="s">
-        <v>134</v>
+        <v>124</v>
+      </c>
+      <c r="H5" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A6" s="5" t="s">
-        <v>29</v>
+      <c r="A6" t="s">
+        <v>27</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="D6" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
       <c r="E6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F6" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="G6" t="s">
-        <v>135</v>
+        <v>125</v>
+      </c>
+      <c r="H6" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C7" t="s">
-        <v>115</v>
+        <v>142</v>
       </c>
       <c r="D7" t="s">
+        <v>111</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
         <v>120</v>
       </c>
-      <c r="E7" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" t="s">
-        <v>129</v>
-      </c>
       <c r="G7" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="D8" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="E8" t="s">
         <v>16</v>
       </c>
       <c r="F8" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D9" t="s">
-        <v>122</v>
-      </c>
-      <c r="E9" t="s">
-        <v>17</v>
+        <v>113</v>
+      </c>
+      <c r="F9" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
-      </c>
-      <c r="E10" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
-        <v>34</v>
-      </c>
       <c r="B11" t="s">
-        <v>45</v>
-      </c>
-      <c r="E11" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
-        <v>46</v>
-      </c>
-      <c r="B12" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fin fin de doc
</commit_message>
<xml_diff>
--- a/src/data/database_projects.xlsx
+++ b/src/data/database_projects.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Valerie\Documents\uni\Uni Lausanne\SP26\géovisualisation\projet\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72EE397B-5BBA-442D-8710-B7CF7D4E49DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80BAF9DA-D979-4704-A348-EF1DAA9DF4CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13276" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13276" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="projects sportsanddev" sheetId="3" r:id="rId1"/>
+    <sheet name="recherches organisations" sheetId="3" r:id="rId1"/>
     <sheet name="database" sheetId="1" r:id="rId2"/>
     <sheet name="attributes" sheetId="2" r:id="rId3"/>
   </sheets>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="148">
   <si>
     <t>region</t>
   </si>
@@ -114,9 +114,6 @@
   </si>
   <si>
     <t>Construction of Infrastructure</t>
-  </si>
-  <si>
-    <t>| to separate several values for 1 category</t>
   </si>
   <si>
     <t>Seniors</t>
@@ -505,18 +502,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -540,10 +531,10 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -833,282 +824,282 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A2" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A2" s="3" t="s">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A3" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A3" s="3" t="s">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A4" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A4" s="3" t="s">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A5" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A5" s="3" t="s">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A6" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A6" s="3" t="s">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A7" s="2" t="s">
         <v>44</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A7" s="3" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1134,57 +1125,57 @@
     <col min="17" max="17" width="17.46484375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="J1" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="M1" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="L1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="M1" s="4" t="s">
+      <c r="N1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="P1" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="N1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="Q1" s="4" t="s">
-        <v>101</v>
+      <c r="Q1" s="3" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.45">
@@ -1192,7 +1183,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C2">
         <v>-1.2833300000000001</v>
@@ -1201,43 +1192,43 @@
         <v>36.816670000000002</v>
       </c>
       <c r="E2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F2" t="s">
         <v>11</v>
       </c>
       <c r="G2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H2" t="s">
+        <v>98</v>
+      </c>
+      <c r="I2" t="s">
         <v>99</v>
       </c>
-      <c r="I2" t="s">
-        <v>100</v>
-      </c>
       <c r="J2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="K2" t="s">
         <v>17</v>
       </c>
       <c r="L2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="M2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="N2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="O2" t="s">
-        <v>137</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>98</v>
+        <v>136</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>97</v>
       </c>
       <c r="Q2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.45">
@@ -1356,9 +1347,7 @@
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="C30" s="1" t="s">
-        <v>29</v>
-      </c>
+      <c r="C30" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1409,28 +1398,28 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C2" t="s">
         <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E2" t="s">
         <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.45">
@@ -1438,25 +1427,25 @@
         <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E3" t="s">
         <v>11</v>
       </c>
       <c r="F3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.45">
@@ -1464,25 +1453,25 @@
         <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E4" t="s">
         <v>12</v>
       </c>
       <c r="F4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.45">
@@ -1490,25 +1479,25 @@
         <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
         <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E5" t="s">
         <v>13</v>
       </c>
       <c r="F5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.45">
@@ -1516,25 +1505,25 @@
         <v>27</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E6" t="s">
         <v>15</v>
       </c>
       <c r="F6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.45">
@@ -1542,22 +1531,22 @@
         <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E7" t="s">
         <v>14</v>
       </c>
       <c r="F7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.45">
@@ -1565,19 +1554,19 @@
         <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E8" t="s">
         <v>16</v>
       </c>
       <c r="F8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.45">
@@ -1585,16 +1574,16 @@
         <v>26</v>
       </c>
       <c r="B9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C9" t="s">
         <v>19</v>
       </c>
       <c r="D9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.45">
@@ -1602,12 +1591,12 @@
         <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>